<commit_message>
correction in format in excel export from tables
</commit_message>
<xml_diff>
--- a/public/assets/templates/template.xlsx
+++ b/public/assets/templates/template.xlsx
@@ -11,59 +11,6 @@
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>AMAT-IA</t>
-  </si>
-  <si>
-    <t>Options</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Articles</t>
-  </si>
-  <si>
-    <t>Progress</t>
-  </si>
-  <si>
-    <t>Tasks</t>
-  </si>
-  <si>
-    <t>Type of rule</t>
-  </si>
-  <si>
-    <t>Number</t>
-  </si>
-  <si>
-    <t>Requirement name</t>
-  </si>
-  <si>
-    <t>Requirement description</t>
-  </si>
-  <si>
-    <t>Date of issue / notification</t>
-  </si>
-  <si>
-    <t>Effective date</t>
-  </si>
-  <si>
-    <t>Renovation date</t>
-  </si>
-  <si>
-    <t>Modified date</t>
-  </si>
-  <si>
-    <t>Aquí van los datos de empresa, logos, tipo de plantilla, etc</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -85,7 +32,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -95,18 +42,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -138,12 +73,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -162,26 +94,26 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>285752</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>142875</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>57151</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>1200152</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>15109</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>171451</xdr:rowOff>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="2 Imagen"/>
+        <xdr:cNvPr id="2" name="1 Imagen"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -194,8 +126,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7829552" y="57151"/>
-          <a:ext cx="914400" cy="914400"/>
+          <a:off x="142875" y="0"/>
+          <a:ext cx="2510659" cy="933450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -529,86 +461,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="10" max="10" width="24.625" customWidth="1"/>
-    <col min="11" max="11" width="25.375" customWidth="1"/>
+    <col min="1" max="1" width="16.25" customWidth="1"/>
+    <col min="2" max="2" width="18.375" customWidth="1"/>
+    <col min="3" max="3" width="17.375" customWidth="1"/>
+    <col min="4" max="4" width="18.125" customWidth="1"/>
+    <col min="5" max="5" width="19.375" customWidth="1"/>
+    <col min="6" max="6" width="17.375" customWidth="1"/>
+    <col min="7" max="7" width="14.625" customWidth="1"/>
+    <col min="9" max="9" width="16.125" customWidth="1"/>
+    <col min="10" max="11" width="20.375" customWidth="1"/>
     <col min="12" max="12" width="19.375" customWidth="1"/>
     <col min="13" max="13" width="16.125" customWidth="1"/>
     <col min="14" max="14" width="15.625" customWidth="1"/>
     <col min="15" max="15" width="17.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="J1" s="4"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="4"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="J3" s="4"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="J4" s="4"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="J5" s="4"/>
-    </row>
-    <row r="6" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
+    <row r="6" s="1" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>